<commit_message>
update nationality extension 1a686a2db8b985f01d1d9fb772dad81e69b44f99
</commit_message>
<xml_diff>
--- a/ig/nr-add-vs-cs-to-id/StructureDefinition-fr-core-observation-resp-rate.xlsx
+++ b/ig/nr-add-vs-cs-to-id/StructureDefinition-fr-core-observation-resp-rate.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-01-29T09:55:21+00:00</t>
+    <t>2024-01-29T12:33:53+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -84,8 +84,7 @@
     <t>Description</t>
   </si>
   <si>
-    <t>Profile of the ObservationResprate profil (described in the HL7 VitalSigns profil) for France | Profilage du profil ObservationResprate (décrit dans le profil HL7 VitaSigns) pour l'usage en France
-This profile specifies the patient's identifiers for France. It uses international extensions (birtplace and nationality) and adds specific French extensions | Ce profil spécifie les identifiants de patient utilisés en France. Il utilise des extensions internationales (birthplace et nationalité) et ajoute des extensions propres à la France.</t>
+    <t>Profile of the ObservationResprate profil (described in the HL7 VitalSigns profil) for France | Profilage du profil ObservationResprate (décrit dans le profil HL7 VitaSigns) pour l'usage en France</t>
   </si>
   <si>
     <t>Purpose</t>

</xml_diff>